<commit_message>
Still 13 to go
</commit_message>
<xml_diff>
--- a/05_coding/atlas/ATLASti_Import_Codebook_MDIMs_v2.xlsx
+++ b/05_coding/atlas/ATLASti_Import_Codebook_MDIMs_v2.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arjen/kDrive/Obsidian/Literature Review MDIM/05_coding/atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5766DBF9-BBEB-8A49-8BE0-6D5D67B7687F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA0A8E2B-A60A-C14E-AAFB-241DDB805DD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="28000" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -2359,7 +2359,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2370,48 +2370,26 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC8CDD3"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC8CDD3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC8CDD3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFC8CDD3"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -2420,10 +2398,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2444,9 +2420,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2484,7 +2460,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -2518,6 +2494,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2552,9 +2529,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2731,12 +2709,12 @@
   <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="55" customWidth="1"/>
-    <col min="2" max="2" width="110" customWidth="1"/>
-    <col min="3" max="5" width="16" customWidth="1"/>
+    <col min="1" max="1" width="55.6640625" customWidth="1"/>
+    <col min="2" max="2" width="110.6640625" customWidth="1"/>
+    <col min="3" max="5" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2753,1622 +2731,1333 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="208" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" ht="384" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" ht="328" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="365" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="192" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+    </row>
+    <row r="12" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+    </row>
+    <row r="13" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>28</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+    </row>
+    <row r="15" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+    </row>
+    <row r="16" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+    </row>
+    <row r="17" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>36</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+    </row>
+    <row r="18" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>38</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+    </row>
+    <row r="19" spans="1:3" ht="288" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>40</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+    </row>
+    <row r="21" spans="1:3" ht="288" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>44</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+    </row>
+    <row r="22" spans="1:3" ht="288" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+    </row>
+    <row r="23" spans="1:3" ht="288" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>48</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" t="s">
         <v>7</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>50</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+    </row>
+    <row r="25" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>52</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" t="s">
         <v>7</v>
       </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="1:5" ht="342" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+    </row>
+    <row r="26" spans="1:3" ht="380" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>54</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" t="s">
         <v>7</v>
       </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
+    </row>
+    <row r="27" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>56</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" t="s">
         <v>7</v>
       </c>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
+    </row>
+    <row r="28" spans="1:3" ht="335" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>58</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" t="s">
         <v>7</v>
       </c>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+    </row>
+    <row r="29" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>60</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" t="s">
         <v>7</v>
       </c>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+    </row>
+    <row r="30" spans="1:3" ht="288" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>62</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+    </row>
+    <row r="31" spans="1:3" ht="335" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>64</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-    </row>
-    <row r="32" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
+    </row>
+    <row r="32" spans="1:3" ht="288" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>66</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" t="s">
         <v>7</v>
       </c>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-    </row>
-    <row r="33" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+    </row>
+    <row r="33" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>68</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" t="s">
         <v>7</v>
       </c>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-    </row>
-    <row r="34" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
+    </row>
+    <row r="34" spans="1:4" ht="256" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>70</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" t="s">
         <v>7</v>
       </c>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-    </row>
-    <row r="35" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A35" s="2" t="s">
+    </row>
+    <row r="35" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>72</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-    </row>
-    <row r="36" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
+    </row>
+    <row r="36" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
         <v>74</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-    </row>
-    <row r="37" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
+    </row>
+    <row r="37" spans="1:4" ht="335" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>76</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" t="s">
         <v>7</v>
       </c>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-    </row>
-    <row r="38" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
+    </row>
+    <row r="38" spans="1:4" ht="192" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>78</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" t="s">
         <v>7</v>
       </c>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-    </row>
-    <row r="39" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
+    </row>
+    <row r="39" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>80</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-    </row>
-    <row r="40" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
+    </row>
+    <row r="40" spans="1:4" ht="272" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>82</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" t="s">
         <v>7</v>
       </c>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-    </row>
-    <row r="41" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
+    </row>
+    <row r="41" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>84</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" t="s">
         <v>7</v>
       </c>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-    </row>
-    <row r="42" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
+    </row>
+    <row r="42" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>86</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" t="s">
         <v>7</v>
       </c>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-    </row>
-    <row r="43" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
+    </row>
+    <row r="43" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
         <v>88</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-    </row>
-    <row r="44" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
+    </row>
+    <row r="44" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>90</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" t="s">
         <v>7</v>
       </c>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-    </row>
-    <row r="45" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
+    </row>
+    <row r="45" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>92</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-    </row>
-    <row r="46" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
+    </row>
+    <row r="46" spans="1:4" ht="208" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>94</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-    </row>
-    <row r="47" spans="1:5" ht="195" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
+    </row>
+    <row r="47" spans="1:4" ht="224" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>96</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-    </row>
-    <row r="48" spans="1:5" ht="165" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
+    </row>
+    <row r="48" spans="1:4" ht="192" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>98</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2" t="s">
+      <c r="D48" t="s">
         <v>100</v>
       </c>
-      <c r="E48" s="2"/>
-    </row>
-    <row r="49" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A49" s="2" t="s">
+    </row>
+    <row r="49" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>101</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2" t="s">
+      <c r="D49" t="s">
         <v>100</v>
       </c>
-      <c r="E49" s="2"/>
-    </row>
-    <row r="50" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
+    </row>
+    <row r="50" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>103</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2" t="s">
+      <c r="D50" t="s">
         <v>100</v>
       </c>
-      <c r="E50" s="2"/>
-    </row>
-    <row r="51" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A51" s="2" t="s">
+    </row>
+    <row r="51" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>105</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2" t="s">
+      <c r="D51" t="s">
         <v>100</v>
       </c>
-      <c r="E51" s="2"/>
-    </row>
-    <row r="52" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
+    </row>
+    <row r="52" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>107</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2" t="s">
+      <c r="D52" t="s">
         <v>100</v>
       </c>
-      <c r="E52" s="2"/>
-    </row>
-    <row r="53" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A53" s="2" t="s">
+    </row>
+    <row r="53" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>109</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2" t="s">
+      <c r="D53" t="s">
         <v>100</v>
       </c>
-      <c r="E53" s="2"/>
-    </row>
-    <row r="54" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A54" s="2" t="s">
+    </row>
+    <row r="54" spans="1:4" ht="192" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>111</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2" t="s">
+      <c r="D54" t="s">
         <v>100</v>
       </c>
-      <c r="E54" s="2"/>
-    </row>
-    <row r="55" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
+    </row>
+    <row r="55" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>113</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2" t="s">
+      <c r="D55" t="s">
         <v>100</v>
       </c>
-      <c r="E55" s="2"/>
-    </row>
-    <row r="56" spans="1:5" ht="225" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
+    </row>
+    <row r="56" spans="1:4" ht="240" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>115</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2" t="s">
+      <c r="D56" t="s">
         <v>100</v>
       </c>
-      <c r="E56" s="2"/>
-    </row>
-    <row r="57" spans="1:5" ht="342" x14ac:dyDescent="0.2">
-      <c r="A57" s="2" t="s">
+    </row>
+    <row r="57" spans="1:4" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>117</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-    </row>
-    <row r="58" spans="1:5" ht="328" x14ac:dyDescent="0.2">
-      <c r="A58" s="2" t="s">
+    </row>
+    <row r="58" spans="1:4" ht="365" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>119</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2" t="s">
+      <c r="D58" t="s">
         <v>100</v>
       </c>
-      <c r="E58" s="2"/>
-    </row>
-    <row r="59" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A59" s="2" t="s">
+    </row>
+    <row r="59" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>121</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2" t="s">
+      <c r="D59" t="s">
         <v>100</v>
       </c>
-      <c r="E59" s="2"/>
-    </row>
-    <row r="60" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A60" s="2" t="s">
+    </row>
+    <row r="60" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
         <v>123</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2" t="s">
+      <c r="D60" t="s">
         <v>100</v>
       </c>
-      <c r="E60" s="2"/>
-    </row>
-    <row r="61" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A61" s="2" t="s">
+    </row>
+    <row r="61" spans="1:4" ht="335" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>125</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2" t="s">
+      <c r="D61" t="s">
         <v>100</v>
       </c>
-      <c r="E61" s="2"/>
-    </row>
-    <row r="62" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A62" s="2" t="s">
+    </row>
+    <row r="62" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>127</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2" t="s">
+      <c r="D62" t="s">
         <v>100</v>
       </c>
-      <c r="E62" s="2"/>
-    </row>
-    <row r="63" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A63" s="2" t="s">
+    </row>
+    <row r="63" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>129</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2" t="s">
+      <c r="D63" t="s">
         <v>100</v>
       </c>
-      <c r="E63" s="2"/>
-    </row>
-    <row r="64" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A64" s="2" t="s">
+    </row>
+    <row r="64" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
         <v>131</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-    </row>
-    <row r="65" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A65" s="2" t="s">
+    </row>
+    <row r="65" spans="1:4" ht="272" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>133</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2" t="s">
+      <c r="D65" t="s">
         <v>100</v>
       </c>
-      <c r="E65" s="2"/>
-    </row>
-    <row r="66" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A66" s="2" t="s">
+    </row>
+    <row r="66" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>135</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2" t="s">
+      <c r="D66" t="s">
         <v>100</v>
       </c>
-      <c r="E66" s="2"/>
-    </row>
-    <row r="67" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A67" s="2" t="s">
+    </row>
+    <row r="67" spans="1:4" ht="335" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
         <v>137</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2" t="s">
+      <c r="D67" t="s">
         <v>100</v>
       </c>
-      <c r="E67" s="2"/>
-    </row>
-    <row r="68" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A68" s="2" t="s">
+    </row>
+    <row r="68" spans="1:4" ht="335" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>139</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2" t="s">
+      <c r="D68" t="s">
         <v>100</v>
       </c>
-      <c r="E68" s="2"/>
-    </row>
-    <row r="69" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A69" s="2" t="s">
+    </row>
+    <row r="69" spans="1:4" ht="192" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
         <v>141</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2" t="s">
+      <c r="D69" t="s">
         <v>100</v>
       </c>
-      <c r="E69" s="2"/>
-    </row>
-    <row r="70" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A70" s="2" t="s">
+    </row>
+    <row r="70" spans="1:4" ht="256" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>143</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2" t="s">
+      <c r="D70" t="s">
         <v>100</v>
       </c>
-      <c r="E70" s="2"/>
-    </row>
-    <row r="71" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
+    </row>
+    <row r="71" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
         <v>145</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2" t="s">
+      <c r="D71" t="s">
         <v>100</v>
       </c>
-      <c r="E71" s="2"/>
-    </row>
-    <row r="72" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A72" s="2" t="s">
+    </row>
+    <row r="72" spans="1:4" ht="256" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
         <v>147</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
-    </row>
-    <row r="73" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A73" s="2" t="s">
+    </row>
+    <row r="73" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>149</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2" t="s">
+      <c r="D73" t="s">
         <v>100</v>
       </c>
-      <c r="E73" s="2"/>
-    </row>
-    <row r="74" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A74" s="2" t="s">
+    </row>
+    <row r="74" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
         <v>151</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2" t="s">
+      <c r="D74" t="s">
         <v>100</v>
       </c>
-      <c r="E74" s="2"/>
-    </row>
-    <row r="75" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A75" s="2" t="s">
+    </row>
+    <row r="75" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
         <v>153</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-    </row>
-    <row r="76" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A76" s="2" t="s">
+    </row>
+    <row r="76" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
         <v>155</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2" t="s">
+      <c r="D76" t="s">
         <v>100</v>
       </c>
-      <c r="E76" s="2"/>
-    </row>
-    <row r="77" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A77" s="2" t="s">
+    </row>
+    <row r="77" spans="1:4" ht="288" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
         <v>157</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2" t="s">
+      <c r="D77" t="s">
         <v>100</v>
       </c>
-      <c r="E77" s="2"/>
-    </row>
-    <row r="78" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A78" s="2" t="s">
+    </row>
+    <row r="78" spans="1:4" ht="320" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
         <v>159</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2" t="s">
+      <c r="D78" t="s">
         <v>100</v>
       </c>
-      <c r="E78" s="2"/>
-    </row>
-    <row r="79" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A79" s="2" t="s">
+    </row>
+    <row r="79" spans="1:4" ht="335" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
         <v>161</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2" t="s">
+      <c r="D79" t="s">
         <v>100</v>
       </c>
-      <c r="E79" s="2"/>
-    </row>
-    <row r="80" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A80" s="2" t="s">
+    </row>
+    <row r="80" spans="1:4" ht="304" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
         <v>163</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2" t="s">
+      <c r="D80" t="s">
         <v>100</v>
       </c>
-      <c r="E80" s="2"/>
-    </row>
-    <row r="81" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A81" s="2" t="s">
+    </row>
+    <row r="81" spans="1:5" ht="208" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>165</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2" t="s">
+      <c r="D81" t="s">
         <v>100</v>
       </c>
-      <c r="E81" s="2"/>
-    </row>
-    <row r="82" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A82" s="2" t="s">
+    </row>
+    <row r="82" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>167</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2" t="s">
+      <c r="D82" t="s">
         <v>100</v>
       </c>
-      <c r="E82" s="2"/>
-    </row>
-    <row r="83" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A83" s="2" t="s">
+    </row>
+    <row r="83" spans="1:5" ht="335" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
         <v>169</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2" t="s">
+      <c r="D83" t="s">
         <v>100</v>
       </c>
-      <c r="E83" s="2"/>
-    </row>
-    <row r="84" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A84" s="2" t="s">
+    </row>
+    <row r="84" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
         <v>171</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2" t="s">
+      <c r="D84" t="s">
         <v>100</v>
       </c>
-      <c r="E84" s="2"/>
-    </row>
-    <row r="85" spans="1:5" ht="225" x14ac:dyDescent="0.2">
-      <c r="A85" s="2" t="s">
+    </row>
+    <row r="85" spans="1:5" ht="256" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
         <v>173</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2" t="s">
+      <c r="D85" t="s">
         <v>100</v>
       </c>
-      <c r="E85" s="2"/>
-    </row>
-    <row r="86" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A86" s="2" t="s">
+    </row>
+    <row r="86" spans="1:5" ht="256" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
         <v>175</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2" t="s">
+      <c r="D86" t="s">
         <v>100</v>
       </c>
-      <c r="E86" s="2"/>
-    </row>
-    <row r="87" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A87" s="2" t="s">
+    </row>
+    <row r="87" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
         <v>177</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2" t="s">
+      <c r="D87" t="s">
         <v>100</v>
       </c>
-      <c r="E87" s="2"/>
-    </row>
-    <row r="88" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A88" s="2" t="s">
+    </row>
+    <row r="88" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
         <v>179</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2" t="s">
+      <c r="D88" t="s">
         <v>100</v>
       </c>
-      <c r="E88" s="2"/>
-    </row>
-    <row r="89" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A89" s="2" t="s">
+    </row>
+    <row r="89" spans="1:5" ht="192" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
         <v>181</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="2" t="s">
+      <c r="E89" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A90" s="2" t="s">
+    <row r="90" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
         <v>184</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2" t="s">
+      <c r="E90" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A91" s="2" t="s">
+    <row r="91" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
         <v>186</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2" t="s">
+      <c r="E91" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="225" x14ac:dyDescent="0.2">
-      <c r="A92" s="2" t="s">
+    <row r="92" spans="1:5" ht="240" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>188</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2" t="s">
+      <c r="E92" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A93" s="2" t="s">
+    <row r="93" spans="1:5" ht="335" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
         <v>190</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2" t="s">
+      <c r="E93" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A94" s="2" t="s">
+    <row r="94" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>192</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
-      <c r="E94" s="2" t="s">
+      <c r="E94" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A95" s="2" t="s">
+    <row r="95" spans="1:5" ht="192" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
         <v>194</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C95" s="2"/>
-      <c r="D95" s="2"/>
-      <c r="E95" s="2" t="s">
+      <c r="E95" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A96" s="2" t="s">
+    <row r="96" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
         <v>196</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C96" s="2"/>
-      <c r="D96" s="2"/>
-      <c r="E96" s="2" t="s">
+      <c r="E96" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A97" s="2" t="s">
+    <row r="97" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
         <v>198</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C97" s="2"/>
-      <c r="D97" s="2"/>
-      <c r="E97" s="2" t="s">
+      <c r="E97" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="210" x14ac:dyDescent="0.2">
-      <c r="A98" s="2" t="s">
+    <row r="98" spans="1:5" ht="240" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
         <v>200</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="C98" s="2"/>
-      <c r="D98" s="2"/>
-      <c r="E98" s="2" t="s">
+      <c r="E98" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A99" s="2" t="s">
+    <row r="99" spans="1:5" ht="335" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
         <v>202</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="C99" s="2"/>
-      <c r="D99" s="2"/>
-      <c r="E99" s="2"/>
-    </row>
-    <row r="100" spans="1:5" ht="328" x14ac:dyDescent="0.2">
-      <c r="A100" s="2" t="s">
+    </row>
+    <row r="100" spans="1:5" ht="350" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>204</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2" t="s">
+      <c r="E100" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A101" s="2" t="s">
+    <row r="101" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
         <v>206</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="C101" s="2"/>
-      <c r="D101" s="2"/>
-      <c r="E101" s="2"/>
-    </row>
-    <row r="102" spans="1:5" ht="180" x14ac:dyDescent="0.2">
-      <c r="A102" s="2" t="s">
+    </row>
+    <row r="102" spans="1:5" ht="192" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>208</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C102" s="2"/>
-      <c r="D102" s="2"/>
-      <c r="E102" s="2" t="s">
+      <c r="E102" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A103" s="2" t="s">
+    <row r="103" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
         <v>210</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="C103" s="2"/>
-      <c r="D103" s="2"/>
-      <c r="E103" s="2" t="s">
+      <c r="E103" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A104" s="2" t="s">
+    <row r="104" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
         <v>212</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C104" s="2"/>
-      <c r="D104" s="2"/>
-      <c r="E104" s="2"/>
-    </row>
-    <row r="105" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A105" s="2" t="s">
+    </row>
+    <row r="105" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
         <v>214</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="C105" s="2"/>
-      <c r="D105" s="2"/>
-      <c r="E105" s="2" t="s">
+      <c r="E105" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A106" s="2" t="s">
+    <row r="106" spans="1:5" ht="288" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
         <v>216</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C106" s="2"/>
-      <c r="D106" s="2"/>
-      <c r="E106" s="2"/>
-    </row>
-    <row r="107" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A107" s="2" t="s">
+    </row>
+    <row r="107" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
         <v>218</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C107" s="2"/>
-      <c r="D107" s="2"/>
-      <c r="E107" s="2" t="s">
+      <c r="E107" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A108" s="2" t="s">
+    <row r="108" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
         <v>220</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C108" s="2"/>
-      <c r="D108" s="2"/>
-      <c r="E108" s="2" t="s">
+      <c r="E108" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="210" x14ac:dyDescent="0.2">
-      <c r="A109" s="2" t="s">
+    <row r="109" spans="1:5" ht="240" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
         <v>222</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="C109" s="2"/>
-      <c r="D109" s="2"/>
-      <c r="E109" s="2"/>
-    </row>
-    <row r="110" spans="1:5" ht="225" x14ac:dyDescent="0.2">
-      <c r="A110" s="2" t="s">
+    </row>
+    <row r="110" spans="1:5" ht="256" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
         <v>224</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C110" s="2"/>
-      <c r="D110" s="2"/>
-      <c r="E110" s="2"/>
-    </row>
-    <row r="111" spans="1:5" ht="240" x14ac:dyDescent="0.2">
-      <c r="A111" s="2" t="s">
+    </row>
+    <row r="111" spans="1:5" ht="256" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
         <v>226</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="C111" s="2"/>
-      <c r="D111" s="2"/>
-      <c r="E111" s="2"/>
-    </row>
-    <row r="112" spans="1:5" ht="165" x14ac:dyDescent="0.2">
-      <c r="A112" s="2" t="s">
+    </row>
+    <row r="112" spans="1:5" ht="176" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
         <v>228</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C112" s="2"/>
-      <c r="D112" s="2"/>
-      <c r="E112" s="2" t="s">
+      <c r="E112" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A113" s="2" t="s">
+    <row r="113" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
         <v>230</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C113" s="2"/>
-      <c r="D113" s="2"/>
-      <c r="E113" s="2" t="s">
+      <c r="E113" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="225" x14ac:dyDescent="0.2">
-      <c r="A114" s="2" t="s">
+    <row r="114" spans="1:5" ht="240" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
         <v>232</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C114" s="2"/>
-      <c r="D114" s="2"/>
-      <c r="E114" s="2" t="s">
+      <c r="E114" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A115" s="2" t="s">
+    <row r="115" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
         <v>234</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="C115" s="2"/>
-      <c r="D115" s="2"/>
-      <c r="E115" s="2" t="s">
+      <c r="E115" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="225" x14ac:dyDescent="0.2">
-      <c r="A116" s="2" t="s">
+    <row r="116" spans="1:5" ht="240" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
         <v>236</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="C116" s="2"/>
-      <c r="D116" s="2"/>
-      <c r="E116" s="2" t="s">
+      <c r="E116" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="255" x14ac:dyDescent="0.2">
-      <c r="A117" s="2" t="s">
+    <row r="117" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
         <v>238</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C117" s="2"/>
-      <c r="D117" s="2"/>
-      <c r="E117" s="2" t="s">
+      <c r="E117" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="165" x14ac:dyDescent="0.2">
-      <c r="A118" s="2" t="s">
+    <row r="118" spans="1:5" ht="176" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
         <v>240</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C118" s="2"/>
-      <c r="D118" s="2"/>
-      <c r="E118" s="2" t="s">
+      <c r="E118" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A119" s="2" t="s">
+    <row r="119" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
         <v>242</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C119" s="2"/>
-      <c r="D119" s="2"/>
-      <c r="E119" s="2"/>
-    </row>
-    <row r="120" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A120" s="2" t="s">
+    </row>
+    <row r="120" spans="1:5" ht="335" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
         <v>244</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C120" s="2"/>
-      <c r="D120" s="2"/>
-      <c r="E120" s="2" t="s">
+      <c r="E120" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A121" s="2" t="s">
+    <row r="121" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
         <v>246</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="C121" s="2"/>
-      <c r="D121" s="2"/>
-      <c r="E121" s="2" t="s">
+      <c r="E121" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A122" s="2" t="s">
+    <row r="122" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
         <v>248</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="C122" s="2"/>
-      <c r="D122" s="2"/>
-      <c r="E122" s="2"/>
-    </row>
-    <row r="123" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A123" s="2" t="s">
+    </row>
+    <row r="123" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
         <v>250</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="C123" s="2"/>
-      <c r="D123" s="2"/>
-      <c r="E123" s="2"/>
-    </row>
-    <row r="124" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A124" s="2" t="s">
+    </row>
+    <row r="124" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
         <v>252</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C124" s="2"/>
-      <c r="D124" s="2"/>
-      <c r="E124" s="2" t="s">
+      <c r="E124" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="300" x14ac:dyDescent="0.2">
-      <c r="A125" s="2" t="s">
+    <row r="125" spans="1:5" ht="320" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
         <v>254</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C125" s="2"/>
-      <c r="D125" s="2"/>
-      <c r="E125" s="2" t="s">
+      <c r="E125" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="126" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A126" s="2" t="s">
+    <row r="126" spans="1:5" ht="335" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
         <v>256</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="C126" s="2"/>
-      <c r="D126" s="2"/>
-      <c r="E126" s="2" t="s">
+      <c r="E126" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="127" spans="1:5" ht="285" x14ac:dyDescent="0.2">
-      <c r="A127" s="2" t="s">
+    <row r="127" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
         <v>258</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C127" s="2"/>
-      <c r="D127" s="2"/>
-      <c r="E127" s="2" t="s">
+      <c r="E127" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="128" spans="1:5" ht="270" x14ac:dyDescent="0.2">
-      <c r="A128" s="2" t="s">
+    <row r="128" spans="1:5" ht="304" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
         <v>260</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="C128" s="2"/>
-      <c r="D128" s="2"/>
-      <c r="E128" s="2"/>
-    </row>
-    <row r="129" spans="1:5" ht="328" x14ac:dyDescent="0.2">
-      <c r="A129" s="2" t="s">
+    </row>
+    <row r="129" spans="1:5" ht="350" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
         <v>262</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C129" s="2"/>
-      <c r="D129" s="2"/>
-      <c r="E129" s="2" t="s">
+      <c r="E129" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="130" spans="1:5" ht="314" x14ac:dyDescent="0.2">
-      <c r="A130" s="2" t="s">
+    <row r="130" spans="1:5" ht="350" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
         <v>264</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C130" s="2"/>
-      <c r="D130" s="2"/>
-      <c r="E130" s="2" t="s">
+      <c r="E130" t="s">
         <v>183</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>